<commit_message>
README: refined the locations tables
</commit_message>
<xml_diff>
--- a/Project-info.xlsx
+++ b/Project-info.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="84">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -63,6 +63,9 @@
     <t xml:space="preserve">RUN, DEV</t>
   </si>
   <si>
+    <t xml:space="preserve">P, D</t>
+  </si>
+  <si>
     <t xml:space="preserve">P</t>
   </si>
   <si>
@@ -129,6 +132,9 @@
     <t xml:space="preserve">D</t>
   </si>
   <si>
+    <t xml:space="preserve">I</t>
+  </si>
+  <si>
     <t xml:space="preserve">JAR, DSRC</t>
   </si>
   <si>
@@ -141,9 +147,6 @@
     <t xml:space="preserve">`deps/&lt;group-id&gt;/&lt;artifact-id&gt;/deps.edn` </t>
   </si>
   <si>
-    <t xml:space="preserve">P, D</t>
-  </si>
-  <si>
     <t xml:space="preserve">RO</t>
   </si>
   <si>
@@ -193,6 +196,9 @@
   </si>
   <si>
     <t xml:space="preserve">Dev+Ops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Itself</t>
   </si>
   <si>
     <t xml:space="preserve">DSRC</t>
@@ -551,7 +557,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="9.34375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.37"/>
@@ -561,7 +567,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="5.8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="4.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="9.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.6"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="9.34"/>
   </cols>
@@ -615,13 +621,13 @@
         <v>13</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -629,13 +635,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>12</v>
@@ -644,13 +650,13 @@
         <v>13</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -658,13 +664,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>12</v>
@@ -673,10 +679,10 @@
         <v>13</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -684,13 +690,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>12</v>
@@ -699,13 +705,13 @@
         <v>13</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -713,13 +719,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>12</v>
@@ -728,33 +734,33 @@
         <v>13</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" s="5" customFormat="true" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -762,13 +768,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>12</v>
@@ -777,56 +783,56 @@
         <v>13</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -834,51 +840,51 @@
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C12" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -886,105 +892,62 @@
         <v>8</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="C14" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C16" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" location="clojure.java.basis/current-basis" display="Current basis"/>
@@ -1030,101 +993,107 @@
         <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>6</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G1" s="8" t="s">
         <v>7</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>58</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G5" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G6" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1158,10 +1127,10 @@
   <sheetData>
     <row r="1" s="16" customFormat="true" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>8</v>
@@ -1169,79 +1138,79 @@
     </row>
     <row r="2" customFormat="false" ht="17.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="32.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="32.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="32.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="17.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>